<commit_message>
feat: Redesign special attendance, add admin broadcast notices, and prepare cloud deployment
</commit_message>
<xml_diff>
--- a/server/samples/College_Master_Import.xlsx
+++ b/server/samples/College_Master_Import.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="29">
   <si>
     <t>Roll_Number</t>
   </si>
@@ -43,19 +43,28 @@
     <t>Total_Percentage</t>
   </si>
   <si>
-    <t>15/10/2024</t>
-  </si>
-  <si>
-    <t>16/10/2024</t>
-  </si>
-  <si>
-    <t>17/10/2024</t>
-  </si>
-  <si>
-    <t>18/10/2024</t>
-  </si>
-  <si>
-    <t>19/10/2024</t>
+    <t>10-Oct-26</t>
+  </si>
+  <si>
+    <t>11-Oct-26</t>
+  </si>
+  <si>
+    <t>17-Oct-26</t>
+  </si>
+  <si>
+    <t>18-Oct-26</t>
+  </si>
+  <si>
+    <t>19-Oct-26</t>
+  </si>
+  <si>
+    <t>20-Oct-26</t>
+  </si>
+  <si>
+    <t>24-Oct-26</t>
+  </si>
+  <si>
+    <t>25-Oct-26</t>
   </si>
   <si>
     <t>101</t>
@@ -77,9 +86,6 @@
   </si>
   <si>
     <t>A</t>
-  </si>
-  <si>
-    <t>P</t>
   </si>
   <si>
     <t>102</t>
@@ -488,7 +494,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -501,10 +507,10 @@
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="18" customWidth="1"/>
-    <col min="11" max="15" width="14" customWidth="1"/>
+    <col min="11" max="18" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -550,28 +556,37 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H2">
         <v>20</v>
@@ -582,43 +597,52 @@
       <c r="J2">
         <v>90</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>2</v>
+      </c>
+      <c r="N2">
+        <v>1</v>
+      </c>
+      <c r="O2">
+        <v>1</v>
+      </c>
+      <c r="P2">
+        <v>1</v>
+      </c>
+      <c r="Q2">
+        <v>1</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" t="s">
         <v>22</v>
       </c>
-      <c r="L2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N2" t="s">
-        <v>22</v>
-      </c>
-      <c r="O2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="F3" t="s">
         <v>23</v>
       </c>
-      <c r="B3" t="s">
+      <c r="G3" t="s">
         <v>24</v>
-      </c>
-      <c r="C3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" t="s">
-        <v>21</v>
       </c>
       <c r="H3">
         <v>20</v>
@@ -629,20 +653,29 @@
       <c r="J3">
         <v>95</v>
       </c>
-      <c r="K3" t="s">
-        <v>22</v>
-      </c>
-      <c r="L3" t="s">
-        <v>22</v>
-      </c>
-      <c r="M3" t="s">
-        <v>22</v>
-      </c>
-      <c r="N3" t="s">
-        <v>22</v>
-      </c>
-      <c r="O3" t="s">
-        <v>22</v>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
+      <c r="N3">
+        <v>1</v>
+      </c>
+      <c r="O3">
+        <v>1</v>
+      </c>
+      <c r="P3">
+        <v>1</v>
+      </c>
+      <c r="Q3">
+        <v>1</v>
+      </c>
+      <c r="R3">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>